<commit_message>
updated functional and non-functional requirements page
</commit_message>
<xml_diff>
--- a/StructureDefinition-ng-appointment.xlsx
+++ b/StructureDefinition-ng-appointment.xlsx
@@ -66,7 +66,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-17T07:55:48+01:00</t>
+    <t>2026-08-17T13:27:53+01:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -629,7 +629,7 @@
     <t>The style of appointment or patient that has been booked in the slot (not service type).</t>
   </si>
   <si>
-    <t>http://terminology.hl7.org/ValueSet/v2-0276</t>
+    <t>http://terminology.hl7.org/ValueSet/v2-0276|3.0.0</t>
   </si>
   <si>
     <t>.code</t>

</xml_diff>